<commit_message>
chore: save attendance exports
</commit_message>
<xml_diff>
--- a/exports/attendance_daily.xlsx
+++ b/exports/attendance_daily.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,20 +441,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Usman Umar Garba</t>
+          <t>Ahmad Umar</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>11:30:27.464215</t>
+          <t>09:15:58.881998</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>kHADIJA MUSA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>09:21:43.246098</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Present</t>
         </is>

</xml_diff>